<commit_message>
Add Sample Type column to sample_mapping template (#59)
* Update sample_file_mapping.csv to add sample type

* Add files via upload

add Sample Type column to sample_mapping Excel template

* Add files via upload

* Add Sample Type column to sample_mapping docs and fix Table 7 image link

- Table 8: add Sample Type row to the data dictionary
- Table 9: add Sample Type column to the example
- Table 7: fix broken image link (Individuals -> individuals casing)

* Remove stray space in CSV header
</commit_message>
<xml_diff>
--- a/resources/seqr_metadata_templates/excel_templates/sample_mapping_template.xlsx
+++ b/resources/seqr_metadata_templates/excel_templates/sample_mapping_template.xlsx
@@ -1,182 +1,160 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edwfor/Documents/Seqr Templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79EEA16B-BE98-BD49-B104-AB254A8C8C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="11580" yWindow="5400" windowWidth="28040" windowHeight="17440"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11580" yWindow="5400" windowWidth="28040" windowHeight="17440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sample_mapping" sheetId="1" r:id="rId1"/>
+    <sheet name="sample_mapping" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Individual ID</t>
-  </si>
-  <si>
-    <t>Sample ID</t>
-  </si>
-  <si>
-    <t>Filenames</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
-    <font>
-      <sz val="12"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="18">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
       <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <i val="1"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -223,19 +201,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -246,19 +224,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -269,19 +247,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="6" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -292,19 +270,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -315,19 +293,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -338,19 +316,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.7999816888943144"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.5999938962981048"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.3999755851924192"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -386,7 +364,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
+        <color theme="4" tint="0.3999755851924192"/>
       </bottom>
       <diagonal/>
     </border>
@@ -472,106 +450,166 @@
     </border>
   </borders>
   <cellStyleXfs count="42">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19"/>
+    <cellStyle name="Good" xfId="6" builtinId="26"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28"/>
+    <cellStyle name="Input" xfId="9" builtinId="20"/>
+    <cellStyle name="Output" xfId="10" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
+    <cellStyle name="Note" xfId="15" builtinId="10"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53"/>
+    <cellStyle name="Total" xfId="17" builtinId="25"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -871,22 +909,39 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Individual ID</t>
+        </is>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Sample ID</t>
+        </is>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Filenames</t>
+        </is>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sample Type</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>